<commit_message>
feat(calculators): implement 16.5.1 method 2 calculations and tests
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.5-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.5-lulucf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4672540D-B5FC-7442-BB35-17D0C3FA44EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E22BFEC-1CB2-F84B-8581-4166296A9384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51220" yWindow="10060" windowWidth="28800" windowHeight="26440" xr2:uid="{A7819E6E-1EF8-024D-B571-91DD1BC0E0B7}"/>
+    <workbookView xWindow="6160" yWindow="1000" windowWidth="45420" windowHeight="26440" xr2:uid="{A7819E6E-1EF8-024D-B571-91DD1BC0E0B7}"/>
   </bookViews>
   <sheets>
     <sheet name="16.5.1.1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="42">
   <si>
     <t>Act</t>
   </si>
@@ -149,9 +149,6 @@
     <t>Years since planting</t>
   </si>
   <si>
-    <t>Hectares to include in removal</t>
-  </si>
-  <si>
     <t>Default stem density</t>
   </si>
   <si>
@@ -159,6 +156,12 @@
   </si>
   <si>
     <t>Actual stem density</t>
+  </si>
+  <si>
+    <t>Custom BAMc</t>
+  </si>
+  <si>
+    <t>Hectares removing carbon</t>
   </si>
 </sst>
 </file>
@@ -206,10 +209,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -553,19 +557,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{304E4C56-4465-6144-908F-761ED9C1F4A0}">
-  <dimension ref="A4:V58"/>
+  <dimension ref="A4:W88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="14.6640625" customWidth="1"/>
     <col min="4" max="5" width="18.1640625" customWidth="1"/>
     <col min="6" max="6" width="16.33203125" customWidth="1"/>
     <col min="7" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="16.5" customWidth="1"/>
-    <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="13" max="13" width="15.6640625" customWidth="1"/>
+    <col min="11" max="12" width="16.5" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>5</v>
       </c>
@@ -578,26 +582,26 @@
       <c r="K4" t="s">
         <v>8</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="G5" t="s">
         <v>5</v>
       </c>
-      <c r="L5" t="s">
-        <v>5</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="M5" t="s">
+        <v>5</v>
+      </c>
+      <c r="S5" t="s">
         <v>18</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <f>44/12</f>
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>4</v>
       </c>
@@ -610,46 +614,47 @@
       <c r="K7" t="s">
         <v>13</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:22" s="5" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B9" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3" t="s">
+    <row r="9" spans="1:23" s="6" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="5"/>
+      <c r="J9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L9" s="3" t="s">
+      <c r="K9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="5"/>
+      <c r="M9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="N9" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:23" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -667,32 +672,32 @@
       <c r="K10" t="s">
         <v>9</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="M10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="N10" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>18</v>
       </c>
-      <c r="O10" s="1" t="s">
+      <c r="P10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>11</v>
       </c>
-      <c r="T10" t="s">
+      <c r="U10" t="s">
         <v>9</v>
       </c>
-      <c r="U10" t="s">
+      <c r="V10" t="s">
         <v>6</v>
       </c>
-      <c r="V10" t="s">
+      <c r="W10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -714,42 +719,42 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <f>VLOOKUP(A11, $R$12:$V$21, 4, FALSE)</f>
+        <f>VLOOKUP(A11, $S$12:$W$21, 4, FALSE)</f>
         <v>0.5</v>
       </c>
       <c r="K11">
-        <f>VLOOKUP(A11, $R$12:$V$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-      <c r="L11">
-        <f>VLOOKUP(A11, $R$12:$V$21, 2, FALSE)</f>
-        <v>5</v>
+        <f>VLOOKUP(A11, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
       </c>
       <c r="M11">
+        <f>VLOOKUP(A11, $S$12:$W$21, 2, FALSE)</f>
         <v>5</v>
       </c>
       <c r="N11">
-        <f>$S$5</f>
+        <v>5</v>
+      </c>
+      <c r="O11">
+        <f>$T$5</f>
         <v>3.6666666666666665</v>
       </c>
-      <c r="O11">
-        <f>N11*G11*E11</f>
+      <c r="P11">
+        <f>O11*G11*E11</f>
         <v>11</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>34</v>
       </c>
-      <c r="T11" t="s">
+      <c r="U11" t="s">
         <v>13</v>
       </c>
-      <c r="U11" t="s">
+      <c r="V11" t="s">
         <v>34</v>
       </c>
-      <c r="V11" t="s">
+      <c r="W11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -764,26 +769,26 @@
         <v>3</v>
       </c>
       <c r="K12">
-        <f t="shared" ref="K12:K13" si="1">VLOOKUP(A12, $R$12:$V$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-      <c r="R12" t="s">
+        <f t="shared" ref="K12:K13" si="1">VLOOKUP(A12, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="S12" t="s">
         <v>21</v>
       </c>
-      <c r="S12">
-        <v>5</v>
-      </c>
       <c r="T12">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U12">
+        <v>10</v>
+      </c>
+      <c r="V12">
         <v>0.5</v>
       </c>
-      <c r="V12">
+      <c r="W12">
         <v>417</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -801,377 +806,1253 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>22</v>
       </c>
-      <c r="S13">
+      <c r="T13">
         <v>45</v>
       </c>
-      <c r="T13">
+      <c r="U13">
         <v>15</v>
       </c>
-      <c r="U13">
+      <c r="V13">
         <v>0.82</v>
       </c>
-      <c r="V13">
+      <c r="W13">
         <v>312</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="R14" t="s">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="S14" t="s">
         <v>23</v>
       </c>
-      <c r="S14">
+      <c r="T14">
         <v>9.6</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <v>8</v>
       </c>
-      <c r="U14">
+      <c r="V14">
         <v>1.2</v>
       </c>
-      <c r="V14">
+      <c r="W14">
         <v>222</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="R15" t="s">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="S15" t="s">
         <v>24</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>4.9000000000000004</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>7</v>
       </c>
-      <c r="U15">
+      <c r="V15">
         <v>0.7</v>
       </c>
-      <c r="V15">
+      <c r="W15">
         <v>1500</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="R16" t="s">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <f t="shared" ref="D16:D58" si="2">IF(C16&lt;=K16, B16,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <f t="shared" ref="E16" si="3">SUM(D16:D18)</f>
+        <v>6</v>
+      </c>
+      <c r="G16">
+        <f>VLOOKUP(A16, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.82</v>
+      </c>
+      <c r="K16">
+        <f>VLOOKUP(A16, $S$12:$W$21, 3, FALSE)</f>
+        <v>15</v>
+      </c>
+      <c r="M16">
+        <f t="shared" ref="M16:M59" si="4">VLOOKUP(A16, $S$12:$W$21, 2, FALSE)</f>
+        <v>45</v>
+      </c>
+      <c r="O16">
+        <f t="shared" ref="O16:O59" si="5">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P16">
+        <f t="shared" ref="P16" si="6">O16*G16*E16</f>
+        <v>18.04</v>
+      </c>
+      <c r="S16" t="s">
         <v>25</v>
       </c>
-      <c r="S16">
+      <c r="T16">
         <v>5.2</v>
       </c>
-      <c r="T16">
+      <c r="U16">
         <v>4</v>
       </c>
-      <c r="U16">
+      <c r="V16">
         <v>1.3</v>
       </c>
-      <c r="V16">
+      <c r="W16">
         <v>740</v>
       </c>
     </row>
-    <row r="17" spans="18:22" x14ac:dyDescent="0.2">
-      <c r="R17" t="s">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="K17">
+        <f>VLOOKUP(A17, $S$12:$W$21, 3, FALSE)</f>
+        <v>15</v>
+      </c>
+      <c r="S17" t="s">
         <v>26</v>
       </c>
-      <c r="S17">
+      <c r="T17">
         <v>1.2</v>
       </c>
-      <c r="T17">
+      <c r="U17">
         <v>4</v>
       </c>
-      <c r="U17">
+      <c r="V17">
         <v>0.3</v>
       </c>
-      <c r="V17" t="s">
+      <c r="W17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="18:22" x14ac:dyDescent="0.2">
-      <c r="R18" t="s">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="K18">
+        <f>VLOOKUP(A18, $S$12:$W$21, 3, FALSE)</f>
+        <v>15</v>
+      </c>
+      <c r="S18" t="s">
         <v>28</v>
       </c>
-      <c r="S18">
+      <c r="T18">
         <v>1.5</v>
       </c>
-      <c r="T18">
-        <v>5</v>
-      </c>
       <c r="U18">
+        <v>5</v>
+      </c>
+      <c r="V18">
         <v>0.3</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="18:22" x14ac:dyDescent="0.2">
-      <c r="R19" t="s">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="S19" t="s">
         <v>29</v>
       </c>
-      <c r="S19">
+      <c r="T19">
         <v>6.7</v>
       </c>
-      <c r="T19">
-        <v>10</v>
-      </c>
       <c r="U19">
+        <v>10</v>
+      </c>
+      <c r="V19">
         <v>0.67</v>
       </c>
-      <c r="V19">
+      <c r="W19">
         <v>250</v>
       </c>
     </row>
-    <row r="20" spans="18:22" x14ac:dyDescent="0.2">
-      <c r="R20" t="s">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="S20" t="s">
         <v>30</v>
       </c>
-      <c r="S20">
+      <c r="T20">
         <v>6</v>
       </c>
-      <c r="T20">
-        <v>10</v>
-      </c>
       <c r="U20">
+        <v>10</v>
+      </c>
+      <c r="V20">
         <v>0.6</v>
       </c>
-      <c r="V20">
+      <c r="W20">
         <v>210</v>
       </c>
     </row>
-    <row r="21" spans="18:22" x14ac:dyDescent="0.2">
-      <c r="R21" t="s">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
+      </c>
+      <c r="D21">
+        <f t="shared" ref="D21" si="7">IF(C21&lt;=K21, B21,0)</f>
+        <v>4</v>
+      </c>
+      <c r="E21">
+        <f t="shared" ref="E21" si="8">SUM(D21:D23)</f>
+        <v>15</v>
+      </c>
+      <c r="G21">
+        <f t="shared" ref="G21:G60" si="9">VLOOKUP(A21, $S$12:$W$21, 4, FALSE)</f>
+        <v>1.2</v>
+      </c>
+      <c r="K21">
+        <f t="shared" ref="K21:K62" si="10">VLOOKUP(A21, $S$12:$W$21, 3, FALSE)</f>
+        <v>8</v>
+      </c>
+      <c r="M21">
+        <f t="shared" ref="M21:M59" si="11">VLOOKUP(A21, $S$12:$W$21, 2, FALSE)</f>
+        <v>9.6</v>
+      </c>
+      <c r="O21">
+        <f t="shared" ref="O21:O59" si="12">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P21">
+        <f t="shared" ref="P21" si="13">O21*G21*E21</f>
+        <v>65.999999999999986</v>
+      </c>
+      <c r="S21" t="s">
         <v>31</v>
       </c>
-      <c r="S21">
+      <c r="T21">
         <v>13</v>
       </c>
-      <c r="T21">
-        <v>10</v>
-      </c>
       <c r="U21">
+        <v>10</v>
+      </c>
+      <c r="V21">
         <v>1.3</v>
       </c>
-      <c r="V21">
+      <c r="W21">
         <v>185</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="34" x14ac:dyDescent="0.2">
-      <c r="A50" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B50" s="2" t="s">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>7</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="K22">
+        <f>VLOOKUP(A22, $S$12:$W$21, 3, FALSE)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23">
+        <v>6</v>
+      </c>
+      <c r="C23">
+        <v>7</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="K23">
+        <f>VLOOKUP(A23, $S$12:$W$21, 3, FALSE)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>7</v>
+      </c>
+      <c r="C26">
+        <v>8</v>
+      </c>
+      <c r="D26">
+        <f t="shared" ref="D26" si="14">IF(C26&lt;=K26, B26,0)</f>
         <v>0</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="E26">
+        <f t="shared" ref="E26" si="15">SUM(D26:D28)</f>
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <f t="shared" ref="G26:G60" si="16">VLOOKUP(A26, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.7</v>
+      </c>
+      <c r="K26">
+        <f t="shared" ref="K26:K62" si="17">VLOOKUP(A26, $S$12:$W$21, 3, FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="M26">
+        <f t="shared" ref="M26:M59" si="18">VLOOKUP(A26, $S$12:$W$21, 2, FALSE)</f>
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="O26">
+        <f t="shared" ref="O26:O59" si="19">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P26">
+        <f t="shared" ref="P26" si="20">O26*G26*E26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27">
+        <v>8</v>
+      </c>
+      <c r="C27">
+        <v>9</v>
+      </c>
+      <c r="D27">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <f>VLOOKUP(A27, $S$12:$W$21, 3, FALSE)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28">
+        <v>9</v>
+      </c>
+      <c r="C28">
+        <v>10</v>
+      </c>
+      <c r="D28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <f>VLOOKUP(A28, $S$12:$W$21, 3, FALSE)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31">
+        <v>10</v>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="D31">
+        <f t="shared" ref="D31" si="21">IF(C31&lt;=K31, B31,0)</f>
+        <v>10</v>
+      </c>
+      <c r="E31">
+        <f t="shared" ref="E31" si="22">SUM(D31:D33)</f>
+        <v>21</v>
+      </c>
+      <c r="G31">
+        <f t="shared" ref="G31:G60" si="23">VLOOKUP(A31, $S$12:$W$21, 4, FALSE)</f>
+        <v>1.3</v>
+      </c>
+      <c r="K31">
+        <f t="shared" ref="K31:K62" si="24">VLOOKUP(A31, $S$12:$W$21, 3, FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="M31">
+        <f t="shared" ref="M31:M59" si="25">VLOOKUP(A31, $S$12:$W$21, 2, FALSE)</f>
+        <v>5.2</v>
+      </c>
+      <c r="O31">
+        <f t="shared" ref="O31:O59" si="26">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P31">
+        <f t="shared" ref="P31" si="27">O31*G31*E31</f>
+        <v>100.1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32">
+        <v>11</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="K32">
+        <f>VLOOKUP(A32, $S$12:$W$21, 3, FALSE)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33">
+        <v>12</v>
+      </c>
+      <c r="C33">
+        <v>5</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <f>VLOOKUP(A33, $S$12:$W$21, 3, FALSE)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36">
+        <v>13</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <f t="shared" ref="D36" si="28">IF(C36&lt;=K36, B36,0)</f>
+        <v>13</v>
+      </c>
+      <c r="E36">
+        <f t="shared" ref="E36" si="29">SUM(D36:D38)</f>
+        <v>42</v>
+      </c>
+      <c r="G36">
+        <f t="shared" ref="G36:G60" si="30">VLOOKUP(A36, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.3</v>
+      </c>
+      <c r="K36">
+        <f t="shared" ref="K36:K62" si="31">VLOOKUP(A36, $S$12:$W$21, 3, FALSE)</f>
+        <v>4</v>
+      </c>
+      <c r="M36">
+        <f t="shared" ref="M36:M59" si="32">VLOOKUP(A36, $S$12:$W$21, 2, FALSE)</f>
+        <v>1.2</v>
+      </c>
+      <c r="O36">
+        <f t="shared" ref="O36:O59" si="33">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P36">
+        <f t="shared" ref="P36" si="34">O36*G36*E36</f>
+        <v>46.199999999999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37">
+        <v>14</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="K37">
+        <f>VLOOKUP(A37, $S$12:$W$21, 3, FALSE)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38">
         <v>15</v>
       </c>
-      <c r="F50" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="C38">
+        <v>3</v>
+      </c>
+      <c r="D38">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="K38">
+        <f>VLOOKUP(A38, $S$12:$W$21, 3, FALSE)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>28</v>
+      </c>
+      <c r="B41">
+        <v>16</v>
+      </c>
+      <c r="C41">
+        <v>5</v>
+      </c>
+      <c r="D41">
+        <f t="shared" ref="D41" si="35">IF(C41&lt;=K41, B41,0)</f>
+        <v>16</v>
+      </c>
+      <c r="E41">
+        <f t="shared" ref="E41" si="36">SUM(D41:D43)</f>
+        <v>51</v>
+      </c>
+      <c r="G41">
+        <f t="shared" ref="G41:G60" si="37">VLOOKUP(A41, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.3</v>
+      </c>
+      <c r="K41">
+        <f t="shared" ref="K41:K62" si="38">VLOOKUP(A41, $S$12:$W$21, 3, FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="M41">
+        <f t="shared" ref="M41:M59" si="39">VLOOKUP(A41, $S$12:$W$21, 2, FALSE)</f>
+        <v>1.5</v>
+      </c>
+      <c r="O41">
+        <f t="shared" ref="O41:O59" si="40">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P41">
+        <f t="shared" ref="P41" si="41">O41*G41*E41</f>
+        <v>56.099999999999994</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>28</v>
+      </c>
+      <c r="B42">
+        <v>17</v>
+      </c>
+      <c r="C42">
+        <v>5</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+      <c r="K42">
+        <f>VLOOKUP(A42, $S$12:$W$21, 3, FALSE)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>28</v>
+      </c>
+      <c r="B43">
+        <v>18</v>
+      </c>
+      <c r="C43">
+        <v>5</v>
+      </c>
+      <c r="D43">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="K43">
+        <f>VLOOKUP(A43, $S$12:$W$21, 3, FALSE)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>29</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46">
+        <f t="shared" ref="D46" si="42">IF(C46&lt;=K46, B46,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E46">
+        <f t="shared" ref="E46" si="43">SUM(D46:D48)</f>
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <f t="shared" ref="G46:G60" si="44">VLOOKUP(A46, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.67</v>
+      </c>
+      <c r="K46">
+        <f t="shared" ref="K46:K62" si="45">VLOOKUP(A46, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="M46">
+        <f t="shared" ref="M46:M59" si="46">VLOOKUP(A46, $S$12:$W$21, 2, FALSE)</f>
+        <v>6.7</v>
+      </c>
+      <c r="O46">
+        <f t="shared" ref="O46:O59" si="47">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P46">
+        <f t="shared" ref="P46" si="48">O46*G46*E46</f>
+        <v>2.4566666666666666</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>29</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47">
+        <v>12</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K47">
+        <f>VLOOKUP(A47, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>29</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48">
+        <v>14</v>
+      </c>
+      <c r="D48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <f>VLOOKUP(A48, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>30</v>
+      </c>
+      <c r="B51">
+        <v>1.5</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <f t="shared" ref="D51" si="49">IF(C51&lt;=K51, B51,0)</f>
+        <v>1.5</v>
+      </c>
+      <c r="E51">
+        <f t="shared" ref="E51" si="50">SUM(D51:D53)</f>
+        <v>7.1999999999999993</v>
+      </c>
+      <c r="G51">
+        <f t="shared" ref="G51:G60" si="51">VLOOKUP(A51, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.6</v>
+      </c>
+      <c r="K51">
+        <f t="shared" ref="K51:K62" si="52">VLOOKUP(A51, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="M51">
+        <f t="shared" ref="M51:M59" si="53">VLOOKUP(A51, $S$12:$W$21, 2, FALSE)</f>
         <v>6</v>
       </c>
-      <c r="H50" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="J50" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K50" t="s">
-        <v>9</v>
-      </c>
-      <c r="L50" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="N50" t="s">
-        <v>18</v>
-      </c>
-      <c r="O50" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>21</v>
-      </c>
-      <c r="B51">
-        <v>3</v>
-      </c>
-      <c r="C51">
-        <v>1</v>
-      </c>
-      <c r="D51">
-        <f>IF(C51&lt;=K51, B51,0)</f>
-        <v>3</v>
-      </c>
-      <c r="E51">
-        <f>SUM(D51:D53)</f>
+      <c r="O51">
+        <f t="shared" ref="O51:O59" si="54">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P51">
+        <f t="shared" ref="P51" si="55">O51*G51*E51</f>
+        <v>15.839999999999996</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>30</v>
+      </c>
+      <c r="B52">
+        <v>2.4</v>
+      </c>
+      <c r="C52">
+        <v>4</v>
+      </c>
+      <c r="D52">
+        <f t="shared" si="2"/>
+        <v>2.4</v>
+      </c>
+      <c r="K52">
+        <f>VLOOKUP(A52, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>30</v>
+      </c>
+      <c r="B53">
+        <v>3.3</v>
+      </c>
+      <c r="C53">
         <v>6</v>
-      </c>
-      <c r="F51">
-        <v>1</v>
-      </c>
-      <c r="G51">
-        <f>VLOOKUP(A51, $R$12:$V$21, 4, FALSE)</f>
-        <v>0.5</v>
-      </c>
-      <c r="H51">
-        <f>VLOOKUP(A51, $R$12:$V$21, 5, FALSE)</f>
-        <v>417</v>
-      </c>
-      <c r="I51">
-        <v>422</v>
-      </c>
-      <c r="J51">
-        <f>G51*(I51/H51)</f>
-        <v>0.50599520383693042</v>
-      </c>
-      <c r="K51">
-        <f>VLOOKUP(A51, $R$12:$V$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-      <c r="L51">
-        <f>VLOOKUP(A51, $R$12:$V$21, 2, FALSE)</f>
-        <v>5</v>
-      </c>
-      <c r="M51">
-        <v>5</v>
-      </c>
-      <c r="N51">
-        <f>$S$5</f>
-        <v>3.6666666666666665</v>
-      </c>
-      <c r="O51">
-        <f>N51*J51*E51</f>
-        <v>11.131894484412468</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>21</v>
-      </c>
-      <c r="B52">
-        <v>3</v>
-      </c>
-      <c r="C52">
-        <v>10</v>
-      </c>
-      <c r="D52">
-        <f t="shared" ref="D52:D53" si="2">IF(C52&lt;=K52, B52,0)</f>
-        <v>3</v>
-      </c>
-      <c r="K52">
-        <f t="shared" ref="K52:K53" si="3">VLOOKUP(A52, $R$12:$V$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>21</v>
-      </c>
-      <c r="B53">
-        <v>4</v>
-      </c>
-      <c r="C53">
-        <v>12</v>
       </c>
       <c r="D53">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="K53">
-        <f t="shared" si="3"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A53, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B56">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C56">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D56">
-        <f>IF(C56&lt;=K56, B56,0)</f>
-        <v>3</v>
+        <f t="shared" ref="D56" si="56">IF(C56&lt;=K56, B56,0)</f>
+        <v>7</v>
       </c>
       <c r="E56">
-        <f>SUM(D56:D58)</f>
-        <v>6</v>
-      </c>
-      <c r="F56">
-        <v>1</v>
+        <f t="shared" ref="E56" si="57">SUM(D56:D58)</f>
+        <v>14</v>
       </c>
       <c r="G56">
-        <f>L56/K56</f>
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="H56">
-        <f>VLOOKUP(A56, $R$12:$V$21, 5, FALSE)</f>
-        <v>417</v>
+        <f t="shared" ref="G56:G60" si="58">VLOOKUP(A56, $S$12:$W$21, 4, FALSE)</f>
+        <v>1.3</v>
       </c>
       <c r="K56">
-        <f>VLOOKUP(A56, $R$12:$V$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-      <c r="L56" s="2">
-        <v>5.5</v>
+        <f t="shared" ref="K56:K62" si="59">VLOOKUP(A56, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
       </c>
       <c r="M56">
-        <v>5</v>
-      </c>
-      <c r="N56">
-        <f>$S$5</f>
+        <f t="shared" ref="M56:M59" si="60">VLOOKUP(A56, $S$12:$W$21, 2, FALSE)</f>
+        <v>13</v>
+      </c>
+      <c r="O56">
+        <f t="shared" ref="O56:O59" si="61">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
-      <c r="O56">
-        <f>N56*G56*E56</f>
-        <v>12.1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P56">
+        <f t="shared" ref="P56" si="62">O56*G56*E56</f>
+        <v>66.733333333333334</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B57">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C57">
         <v>10</v>
       </c>
       <c r="D57">
-        <f t="shared" ref="D57:D58" si="4">IF(C57&lt;=K57, B57,0)</f>
-        <v>3</v>
+        <f t="shared" si="2"/>
+        <v>7</v>
       </c>
       <c r="K57">
-        <f t="shared" ref="K57:K58" si="5">VLOOKUP(A57, $R$12:$V$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A57, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B58">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C58">
         <v>12</v>
       </c>
       <c r="D58">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K58">
-        <f t="shared" si="5"/>
-        <v>10</v>
+        <f>VLOOKUP(A58, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G70" t="s">
+        <v>6</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I70" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J70" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="K70" t="s">
+        <v>9</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="M70" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="O70" t="s">
+        <v>18</v>
+      </c>
+      <c r="P70" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>21</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71">
+        <v>1</v>
+      </c>
+      <c r="D71">
+        <f>IF(C71&lt;=K71, B71,0)</f>
+        <v>3</v>
+      </c>
+      <c r="E71">
+        <f>SUM(D71:D73)</f>
+        <v>6</v>
+      </c>
+      <c r="F71">
+        <v>1</v>
+      </c>
+      <c r="G71">
+        <f>VLOOKUP(A71, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.5</v>
+      </c>
+      <c r="H71">
+        <f>VLOOKUP(A71, $S$12:$W$21, 5, FALSE)</f>
+        <v>417</v>
+      </c>
+      <c r="I71" s="2">
+        <v>422</v>
+      </c>
+      <c r="J71">
+        <f>G71*(I71/H71)</f>
+        <v>0.50599520383693042</v>
+      </c>
+      <c r="K71">
+        <f>VLOOKUP(A71, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="M71">
+        <f>IF(ISBLANK(L71),VLOOKUP(A71, $S$12:$W$21, 2, FALSE),L71)</f>
+        <v>5</v>
+      </c>
+      <c r="N71">
+        <v>5</v>
+      </c>
+      <c r="O71">
+        <f>$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P71">
+        <f>O71*J71*E71</f>
+        <v>11.131894484412468</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>21</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72">
+        <v>10</v>
+      </c>
+      <c r="D72">
+        <f t="shared" ref="D72:D73" si="63">IF(C72&lt;=K72, B72,0)</f>
+        <v>3</v>
+      </c>
+      <c r="K72">
+        <f t="shared" ref="K72:K73" si="64">VLOOKUP(A72, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>21</v>
+      </c>
+      <c r="B73">
+        <v>4</v>
+      </c>
+      <c r="C73">
+        <v>12</v>
+      </c>
+      <c r="D73">
+        <f t="shared" si="63"/>
+        <v>0</v>
+      </c>
+      <c r="K73">
+        <f t="shared" si="64"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>21</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76">
+        <v>1</v>
+      </c>
+      <c r="D76">
+        <f>IF(C76&lt;=K76, B76,0)</f>
+        <v>3</v>
+      </c>
+      <c r="E76">
+        <f>SUM(D76:D78)</f>
+        <v>6</v>
+      </c>
+      <c r="F76">
+        <v>1</v>
+      </c>
+      <c r="G76">
+        <f>M76/K76</f>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="H76">
+        <f>VLOOKUP(A76, $S$12:$W$21, 5, FALSE)</f>
+        <v>417</v>
+      </c>
+      <c r="K76">
+        <f>VLOOKUP(A76, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="L76" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="M76">
+        <f t="shared" ref="M76" si="65">IF(ISBLANK(L76),VLOOKUP(A76, $S$12:$W$21, 2, FALSE),L76)</f>
+        <v>5.5</v>
+      </c>
+      <c r="N76">
+        <v>5</v>
+      </c>
+      <c r="O76">
+        <f>$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P76">
+        <f>O76*G76*E76</f>
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>21</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77">
+        <v>10</v>
+      </c>
+      <c r="D77">
+        <f t="shared" ref="D77:D78" si="66">IF(C77&lt;=K77, B77,0)</f>
+        <v>3</v>
+      </c>
+      <c r="K77">
+        <f t="shared" ref="K77:K78" si="67">VLOOKUP(A77, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>21</v>
+      </c>
+      <c r="B78">
+        <v>4</v>
+      </c>
+      <c r="C78">
+        <v>12</v>
+      </c>
+      <c r="D78">
+        <f t="shared" si="66"/>
+        <v>0</v>
+      </c>
+      <c r="K78">
+        <f t="shared" si="67"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>31</v>
+      </c>
+      <c r="B81">
+        <v>3</v>
+      </c>
+      <c r="C81">
+        <v>1</v>
+      </c>
+      <c r="D81">
+        <f>IF(C81&lt;=K81, B81,0)</f>
+        <v>3</v>
+      </c>
+      <c r="E81">
+        <f>SUM(D81:D83)</f>
+        <v>6</v>
+      </c>
+      <c r="F81">
+        <v>1</v>
+      </c>
+      <c r="G81">
+        <f>VLOOKUP(A81, $S$12:$W$21, 4, FALSE)</f>
+        <v>1.3</v>
+      </c>
+      <c r="H81">
+        <f>VLOOKUP(A81, $S$12:$W$21, 5, FALSE)</f>
+        <v>185</v>
+      </c>
+      <c r="I81" s="2">
+        <v>410</v>
+      </c>
+      <c r="J81">
+        <f>G81*(I81/H81)</f>
+        <v>2.8810810810810814</v>
+      </c>
+      <c r="K81">
+        <f>VLOOKUP(A81, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="M81">
+        <f>IF(ISBLANK(L81),VLOOKUP(A81, $S$12:$W$21, 2, FALSE),L81)</f>
+        <v>13</v>
+      </c>
+      <c r="N81">
+        <v>5</v>
+      </c>
+      <c r="O81">
+        <f>$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P81">
+        <f>O81*J81*E81</f>
+        <v>63.383783783783784</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>31</v>
+      </c>
+      <c r="B82">
+        <v>3</v>
+      </c>
+      <c r="C82">
+        <v>10</v>
+      </c>
+      <c r="D82">
+        <f t="shared" ref="D82:D83" si="68">IF(C82&lt;=K82, B82,0)</f>
+        <v>3</v>
+      </c>
+      <c r="K82">
+        <f t="shared" ref="K82:K83" si="69">VLOOKUP(A82, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>31</v>
+      </c>
+      <c r="B83">
+        <v>4</v>
+      </c>
+      <c r="C83">
+        <v>12</v>
+      </c>
+      <c r="D83">
+        <f t="shared" si="68"/>
+        <v>0</v>
+      </c>
+      <c r="K83">
+        <f t="shared" si="69"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>24</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="D86">
+        <f>IF(C86&lt;=K86, B86,0)</f>
+        <v>3</v>
+      </c>
+      <c r="E86">
+        <f>SUM(D86:D88)</f>
+        <v>3</v>
+      </c>
+      <c r="F86">
+        <v>1</v>
+      </c>
+      <c r="G86">
+        <f>M86/K86</f>
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="H86">
+        <f>VLOOKUP(A86, $S$12:$W$21, 5, FALSE)</f>
+        <v>1500</v>
+      </c>
+      <c r="K86">
+        <f>VLOOKUP(A86, $S$12:$W$21, 3, FALSE)</f>
+        <v>7</v>
+      </c>
+      <c r="L86" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="M86">
+        <f t="shared" ref="M86" si="70">IF(ISBLANK(L86),VLOOKUP(A86, $S$12:$W$21, 2, FALSE),L86)</f>
+        <v>4.5</v>
+      </c>
+      <c r="N86">
+        <v>5</v>
+      </c>
+      <c r="O86">
+        <f>$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P86">
+        <f>O86*G86*E86</f>
+        <v>7.0714285714285712</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>24</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87">
+        <v>10</v>
+      </c>
+      <c r="D87">
+        <f t="shared" ref="D87:D88" si="71">IF(C87&lt;=K87, B87,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K87">
+        <f t="shared" ref="K87:K88" si="72">VLOOKUP(A87, $S$12:$W$21, 3, FALSE)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>24</v>
+      </c>
+      <c r="B88">
+        <v>4</v>
+      </c>
+      <c r="C88">
+        <v>12</v>
+      </c>
+      <c r="D88">
+        <f t="shared" si="71"/>
+        <v>0</v>
+      </c>
+      <c r="K88">
+        <f t="shared" si="72"/>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(calculators): finish 16.5.1.3 and 4, including method 2 support
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.5-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.5-lulucf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E22BFEC-1CB2-F84B-8581-4166296A9384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1DA4E4-3AE5-6C4C-A792-58CF127D8BD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6160" yWindow="1000" windowWidth="45420" windowHeight="26440" xr2:uid="{A7819E6E-1EF8-024D-B571-91DD1BC0E0B7}"/>
+    <workbookView xWindow="51220" yWindow="11100" windowWidth="28800" windowHeight="26440" xr2:uid="{A7819E6E-1EF8-024D-B571-91DD1BC0E0B7}"/>
   </bookViews>
   <sheets>
     <sheet name="16.5.1.1" sheetId="1" r:id="rId1"/>
@@ -86,9 +86,6 @@
     <t>t</t>
   </si>
   <si>
-    <t>Age of crop at time of clearing</t>
-  </si>
-  <si>
     <t>Biomass stock at maturity</t>
   </si>
   <si>
@@ -143,9 +140,6 @@
     <t>tC / ha / yr</t>
   </si>
   <si>
-    <t>tclearing</t>
-  </si>
-  <si>
     <t>Years since planting</t>
   </si>
   <si>
@@ -162,6 +156,12 @@
   </si>
   <si>
     <t>Hectares removing carbon</t>
+  </si>
+  <si>
+    <t>ELUc</t>
+  </si>
+  <si>
+    <t>BAMc for 16.5.1.4</t>
   </si>
 </sst>
 </file>
@@ -565,8 +565,7 @@
     <col min="6" max="6" width="16.33203125" customWidth="1"/>
     <col min="7" max="10" width="17" customWidth="1"/>
     <col min="11" max="12" width="16.5" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" customWidth="1"/>
+    <col min="13" max="14" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
@@ -594,7 +593,7 @@
         <v>5</v>
       </c>
       <c r="S5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T5">
         <f>44/12</f>
@@ -623,10 +622,10 @@
         <v>1</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="4" t="s">
@@ -636,26 +635,24 @@
         <v>7</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="N9" s="4" t="s">
         <v>16</v>
       </c>
+      <c r="N9" s="4"/>
     </row>
     <row r="10" spans="1:23" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>0</v>
@@ -675,14 +672,15 @@
       <c r="M10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N10" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="N10" s="2"/>
       <c r="O10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="P10" s="1" t="s">
-        <v>19</v>
+      <c r="Q10" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="T10" t="s">
         <v>11</v>
@@ -694,12 +692,12 @@
         <v>6</v>
       </c>
       <c r="W10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -730,9 +728,6 @@
         <f>VLOOKUP(A11, $S$12:$W$21, 2, FALSE)</f>
         <v>5</v>
       </c>
-      <c r="N11">
-        <v>5</v>
-      </c>
       <c r="O11">
         <f>$T$5</f>
         <v>3.6666666666666665</v>
@@ -741,22 +736,26 @@
         <f>O11*G11*E11</f>
         <v>11</v>
       </c>
+      <c r="Q11">
+        <f>O11*M11*F11</f>
+        <v>18.333333333333332</v>
+      </c>
       <c r="T11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U11" t="s">
         <v>13</v>
       </c>
       <c r="V11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="W11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>3</v>
@@ -769,11 +768,11 @@
         <v>3</v>
       </c>
       <c r="K12">
-        <f t="shared" ref="K12:K13" si="1">VLOOKUP(A12, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A12, $S$12:$W$21, 3, FALSE)</f>
         <v>10</v>
       </c>
       <c r="S12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="T12">
         <v>5</v>
@@ -790,7 +789,7 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <v>4</v>
@@ -803,11 +802,11 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP(A13, $S$12:$W$21, 3, FALSE)</f>
         <v>10</v>
       </c>
       <c r="S13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="T13">
         <v>45</v>
@@ -824,7 +823,7 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="S14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="T14">
         <v>9.6</v>
@@ -841,7 +840,7 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="S15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="T15">
         <v>4.9000000000000004</v>
@@ -858,7 +857,7 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -867,12 +866,15 @@
         <v>1</v>
       </c>
       <c r="D16">
-        <f t="shared" ref="D16:D58" si="2">IF(C16&lt;=K16, B16,0)</f>
+        <f t="shared" ref="D16:D58" si="1">IF(C16&lt;=K16, B16,0)</f>
         <v>1</v>
       </c>
       <c r="E16">
-        <f t="shared" ref="E16" si="3">SUM(D16:D18)</f>
+        <f t="shared" ref="E16" si="2">SUM(D16:D18)</f>
         <v>6</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
       </c>
       <c r="G16">
         <f>VLOOKUP(A16, $S$12:$W$21, 4, FALSE)</f>
@@ -883,19 +885,23 @@
         <v>15</v>
       </c>
       <c r="M16">
-        <f t="shared" ref="M16:M59" si="4">VLOOKUP(A16, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A16, $S$12:$W$21, 2, FALSE)</f>
         <v>45</v>
       </c>
       <c r="O16">
-        <f t="shared" ref="O16:O59" si="5">$T$5</f>
+        <f t="shared" ref="O16:O59" si="3">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P16">
-        <f t="shared" ref="P16" si="6">O16*G16*E16</f>
+        <f>O16*G16*E16</f>
         <v>18.04</v>
       </c>
+      <c r="Q16">
+        <f>O16*M16*F16</f>
+        <v>0</v>
+      </c>
       <c r="S16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="T16">
         <v>5.2</v>
@@ -912,7 +918,7 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -921,7 +927,7 @@
         <v>1</v>
       </c>
       <c r="D17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="K17">
@@ -929,7 +935,7 @@
         <v>15</v>
       </c>
       <c r="S17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="T17">
         <v>1.2</v>
@@ -941,12 +947,12 @@
         <v>0.3</v>
       </c>
       <c r="W17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -955,7 +961,7 @@
         <v>1</v>
       </c>
       <c r="D18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="K18">
@@ -963,7 +969,7 @@
         <v>15</v>
       </c>
       <c r="S18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="T18">
         <v>1.5</v>
@@ -975,12 +981,12 @@
         <v>0.3</v>
       </c>
       <c r="W18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="S19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T19">
         <v>6.7</v>
@@ -997,7 +1003,7 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="S20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="T20">
         <v>6</v>
@@ -1014,7 +1020,7 @@
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21">
         <v>4</v>
@@ -1023,35 +1029,42 @@
         <v>7</v>
       </c>
       <c r="D21">
-        <f t="shared" ref="D21" si="7">IF(C21&lt;=K21, B21,0)</f>
+        <f t="shared" ref="D21" si="4">IF(C21&lt;=K21, B21,0)</f>
         <v>4</v>
       </c>
       <c r="E21">
-        <f t="shared" ref="E21" si="8">SUM(D21:D23)</f>
+        <f t="shared" ref="E21" si="5">SUM(D21:D23)</f>
         <v>15</v>
       </c>
+      <c r="F21">
+        <v>2.5</v>
+      </c>
       <c r="G21">
-        <f t="shared" ref="G21:G60" si="9">VLOOKUP(A21, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A21, $S$12:$W$21, 4, FALSE)</f>
         <v>1.2</v>
       </c>
       <c r="K21">
-        <f t="shared" ref="K21:K62" si="10">VLOOKUP(A21, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A21, $S$12:$W$21, 3, FALSE)</f>
         <v>8</v>
       </c>
       <c r="M21">
-        <f t="shared" ref="M21:M59" si="11">VLOOKUP(A21, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A21, $S$12:$W$21, 2, FALSE)</f>
         <v>9.6</v>
       </c>
       <c r="O21">
-        <f t="shared" ref="O21:O59" si="12">$T$5</f>
+        <f t="shared" ref="O21:O59" si="6">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P21">
-        <f t="shared" ref="P21" si="13">O21*G21*E21</f>
+        <f>O21*G21*E21</f>
         <v>65.999999999999986</v>
       </c>
+      <c r="Q21">
+        <f>O21*M21*F21</f>
+        <v>87.999999999999986</v>
+      </c>
       <c r="S21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T21">
         <v>13</v>
@@ -1068,7 +1081,7 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22">
         <v>5</v>
@@ -1077,7 +1090,7 @@
         <v>7</v>
       </c>
       <c r="D22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="K22">
@@ -1087,7 +1100,7 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>6</v>
@@ -1096,7 +1109,7 @@
         <v>7</v>
       </c>
       <c r="D23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="K23">
@@ -1106,7 +1119,7 @@
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26">
         <v>7</v>
@@ -1115,37 +1128,44 @@
         <v>8</v>
       </c>
       <c r="D26">
-        <f t="shared" ref="D26" si="14">IF(C26&lt;=K26, B26,0)</f>
+        <f t="shared" ref="D26" si="7">IF(C26&lt;=K26, B26,0)</f>
         <v>0</v>
       </c>
       <c r="E26">
-        <f t="shared" ref="E26" si="15">SUM(D26:D28)</f>
+        <f t="shared" ref="E26" si="8">SUM(D26:D28)</f>
         <v>0</v>
       </c>
+      <c r="F26">
+        <v>5</v>
+      </c>
       <c r="G26">
-        <f t="shared" ref="G26:G60" si="16">VLOOKUP(A26, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A26, $S$12:$W$21, 4, FALSE)</f>
         <v>0.7</v>
       </c>
       <c r="K26">
-        <f t="shared" ref="K26:K62" si="17">VLOOKUP(A26, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A26, $S$12:$W$21, 3, FALSE)</f>
         <v>7</v>
       </c>
       <c r="M26">
-        <f t="shared" ref="M26:M59" si="18">VLOOKUP(A26, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A26, $S$12:$W$21, 2, FALSE)</f>
         <v>4.9000000000000004</v>
       </c>
       <c r="O26">
-        <f t="shared" ref="O26:O59" si="19">$T$5</f>
+        <f t="shared" ref="O26:O59" si="9">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P26">
-        <f t="shared" ref="P26" si="20">O26*G26*E26</f>
+        <f>O26*G26*E26</f>
         <v>0</v>
+      </c>
+      <c r="Q26">
+        <f>O26*M26*F26</f>
+        <v>89.833333333333343</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27">
         <v>8</v>
@@ -1154,7 +1174,7 @@
         <v>9</v>
       </c>
       <c r="D27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K27">
@@ -1164,7 +1184,7 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28">
         <v>9</v>
@@ -1173,7 +1193,7 @@
         <v>10</v>
       </c>
       <c r="D28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K28">
@@ -1183,7 +1203,7 @@
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B31">
         <v>10</v>
@@ -1192,37 +1212,44 @@
         <v>3</v>
       </c>
       <c r="D31">
-        <f t="shared" ref="D31" si="21">IF(C31&lt;=K31, B31,0)</f>
+        <f t="shared" ref="D31" si="10">IF(C31&lt;=K31, B31,0)</f>
         <v>10</v>
       </c>
       <c r="E31">
-        <f t="shared" ref="E31" si="22">SUM(D31:D33)</f>
+        <f t="shared" ref="E31" si="11">SUM(D31:D33)</f>
         <v>21</v>
       </c>
+      <c r="F31">
+        <v>20</v>
+      </c>
       <c r="G31">
-        <f t="shared" ref="G31:G60" si="23">VLOOKUP(A31, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A31, $S$12:$W$21, 4, FALSE)</f>
         <v>1.3</v>
       </c>
       <c r="K31">
-        <f t="shared" ref="K31:K62" si="24">VLOOKUP(A31, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A31, $S$12:$W$21, 3, FALSE)</f>
         <v>4</v>
       </c>
       <c r="M31">
-        <f t="shared" ref="M31:M59" si="25">VLOOKUP(A31, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A31, $S$12:$W$21, 2, FALSE)</f>
         <v>5.2</v>
       </c>
       <c r="O31">
-        <f t="shared" ref="O31:O59" si="26">$T$5</f>
+        <f t="shared" ref="O31:O59" si="12">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P31">
-        <f t="shared" ref="P31" si="27">O31*G31*E31</f>
+        <f>O31*G31*E31</f>
         <v>100.1</v>
+      </c>
+      <c r="Q31">
+        <f>O31*M31*F31</f>
+        <v>381.33333333333331</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B32">
         <v>11</v>
@@ -1231,7 +1258,7 @@
         <v>4</v>
       </c>
       <c r="D32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="K32">
@@ -1239,9 +1266,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B33">
         <v>12</v>
@@ -1250,7 +1277,7 @@
         <v>5</v>
       </c>
       <c r="D33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K33">
@@ -1258,9 +1285,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36">
         <v>13</v>
@@ -1269,37 +1296,44 @@
         <v>1</v>
       </c>
       <c r="D36">
-        <f t="shared" ref="D36" si="28">IF(C36&lt;=K36, B36,0)</f>
+        <f t="shared" ref="D36" si="13">IF(C36&lt;=K36, B36,0)</f>
         <v>13</v>
       </c>
       <c r="E36">
-        <f t="shared" ref="E36" si="29">SUM(D36:D38)</f>
+        <f t="shared" ref="E36" si="14">SUM(D36:D38)</f>
         <v>42</v>
       </c>
+      <c r="F36">
+        <v>0.3</v>
+      </c>
       <c r="G36">
-        <f t="shared" ref="G36:G60" si="30">VLOOKUP(A36, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A36, $S$12:$W$21, 4, FALSE)</f>
         <v>0.3</v>
       </c>
       <c r="K36">
-        <f t="shared" ref="K36:K62" si="31">VLOOKUP(A36, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A36, $S$12:$W$21, 3, FALSE)</f>
         <v>4</v>
       </c>
       <c r="M36">
-        <f t="shared" ref="M36:M59" si="32">VLOOKUP(A36, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A36, $S$12:$W$21, 2, FALSE)</f>
         <v>1.2</v>
       </c>
       <c r="O36">
-        <f t="shared" ref="O36:O59" si="33">$T$5</f>
+        <f t="shared" ref="O36:O59" si="15">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P36">
-        <f t="shared" ref="P36" si="34">O36*G36*E36</f>
+        <f>O36*G36*E36</f>
         <v>46.199999999999996</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q36">
+        <f>O36*M36*F36</f>
+        <v>1.3199999999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B37">
         <v>14</v>
@@ -1308,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="D37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="K37">
@@ -1316,9 +1350,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B38">
         <v>15</v>
@@ -1327,7 +1361,7 @@
         <v>3</v>
       </c>
       <c r="D38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="K38">
@@ -1335,9 +1369,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41">
         <v>16</v>
@@ -1346,37 +1380,44 @@
         <v>5</v>
       </c>
       <c r="D41">
-        <f t="shared" ref="D41" si="35">IF(C41&lt;=K41, B41,0)</f>
+        <f t="shared" ref="D41" si="16">IF(C41&lt;=K41, B41,0)</f>
         <v>16</v>
       </c>
       <c r="E41">
-        <f t="shared" ref="E41" si="36">SUM(D41:D43)</f>
+        <f t="shared" ref="E41" si="17">SUM(D41:D43)</f>
         <v>51</v>
       </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
       <c r="G41">
-        <f t="shared" ref="G41:G60" si="37">VLOOKUP(A41, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A41, $S$12:$W$21, 4, FALSE)</f>
         <v>0.3</v>
       </c>
       <c r="K41">
-        <f t="shared" ref="K41:K62" si="38">VLOOKUP(A41, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A41, $S$12:$W$21, 3, FALSE)</f>
         <v>5</v>
       </c>
       <c r="M41">
-        <f t="shared" ref="M41:M59" si="39">VLOOKUP(A41, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A41, $S$12:$W$21, 2, FALSE)</f>
         <v>1.5</v>
       </c>
       <c r="O41">
-        <f t="shared" ref="O41:O59" si="40">$T$5</f>
+        <f t="shared" ref="O41:O59" si="18">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P41">
-        <f t="shared" ref="P41" si="41">O41*G41*E41</f>
+        <f>O41*G41*E41</f>
         <v>56.099999999999994</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q41">
+        <f>O41*M41*F41</f>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B42">
         <v>17</v>
@@ -1385,7 +1426,7 @@
         <v>5</v>
       </c>
       <c r="D42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="K42">
@@ -1393,9 +1434,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B43">
         <v>18</v>
@@ -1404,7 +1445,7 @@
         <v>5</v>
       </c>
       <c r="D43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="K43">
@@ -1412,9 +1453,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -1423,37 +1464,44 @@
         <v>1</v>
       </c>
       <c r="D46">
-        <f t="shared" ref="D46" si="42">IF(C46&lt;=K46, B46,0)</f>
+        <f t="shared" ref="D46" si="19">IF(C46&lt;=K46, B46,0)</f>
         <v>1</v>
       </c>
       <c r="E46">
-        <f t="shared" ref="E46" si="43">SUM(D46:D48)</f>
-        <v>1</v>
+        <f t="shared" ref="E46" si="20">SUM(D46:D48)</f>
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>4</v>
       </c>
       <c r="G46">
-        <f t="shared" ref="G46:G60" si="44">VLOOKUP(A46, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A46, $S$12:$W$21, 4, FALSE)</f>
         <v>0.67</v>
       </c>
       <c r="K46">
-        <f t="shared" ref="K46:K62" si="45">VLOOKUP(A46, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A46, $S$12:$W$21, 3, FALSE)</f>
         <v>10</v>
       </c>
       <c r="M46">
-        <f t="shared" ref="M46:M59" si="46">VLOOKUP(A46, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A46, $S$12:$W$21, 2, FALSE)</f>
         <v>6.7</v>
       </c>
       <c r="O46">
-        <f t="shared" ref="O46:O59" si="47">$T$5</f>
+        <f t="shared" ref="O46:O59" si="21">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P46">
-        <f t="shared" ref="P46" si="48">O46*G46*E46</f>
+        <f>O46*G46*E46</f>
         <v>2.4566666666666666</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q46">
+        <f>O46*M46*F46</f>
+        <v>98.266666666666666</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B47">
         <v>1</v>
@@ -1462,7 +1510,7 @@
         <v>12</v>
       </c>
       <c r="D47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K47">
@@ -1470,9 +1518,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B48">
         <v>1</v>
@@ -1481,7 +1529,7 @@
         <v>14</v>
       </c>
       <c r="D48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K48">
@@ -1489,9 +1537,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B51">
         <v>1.5</v>
@@ -1500,37 +1548,44 @@
         <v>2</v>
       </c>
       <c r="D51">
-        <f t="shared" ref="D51" si="49">IF(C51&lt;=K51, B51,0)</f>
+        <f t="shared" ref="D51" si="22">IF(C51&lt;=K51, B51,0)</f>
         <v>1.5</v>
       </c>
       <c r="E51">
-        <f t="shared" ref="E51" si="50">SUM(D51:D53)</f>
+        <f t="shared" ref="E51" si="23">SUM(D51:D53)</f>
         <v>7.1999999999999993</v>
       </c>
+      <c r="F51">
+        <v>2</v>
+      </c>
       <c r="G51">
-        <f t="shared" ref="G51:G60" si="51">VLOOKUP(A51, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A51, $S$12:$W$21, 4, FALSE)</f>
         <v>0.6</v>
       </c>
       <c r="K51">
-        <f t="shared" ref="K51:K62" si="52">VLOOKUP(A51, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A51, $S$12:$W$21, 3, FALSE)</f>
         <v>10</v>
       </c>
       <c r="M51">
-        <f t="shared" ref="M51:M59" si="53">VLOOKUP(A51, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A51, $S$12:$W$21, 2, FALSE)</f>
         <v>6</v>
       </c>
       <c r="O51">
-        <f t="shared" ref="O51:O59" si="54">$T$5</f>
+        <f t="shared" ref="O51:O59" si="24">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P51">
-        <f t="shared" ref="P51" si="55">O51*G51*E51</f>
+        <f>O51*G51*E51</f>
         <v>15.839999999999996</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q51">
+        <f>O51*M51*F51</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B52">
         <v>2.4</v>
@@ -1539,7 +1594,7 @@
         <v>4</v>
       </c>
       <c r="D52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>2.4</v>
       </c>
       <c r="K52">
@@ -1547,9 +1602,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B53">
         <v>3.3</v>
@@ -1558,7 +1613,7 @@
         <v>6</v>
       </c>
       <c r="D53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3.3</v>
       </c>
       <c r="K53">
@@ -1566,9 +1621,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B56">
         <v>7</v>
@@ -1577,37 +1632,44 @@
         <v>8</v>
       </c>
       <c r="D56">
-        <f t="shared" ref="D56" si="56">IF(C56&lt;=K56, B56,0)</f>
+        <f t="shared" ref="D56" si="25">IF(C56&lt;=K56, B56,0)</f>
         <v>7</v>
       </c>
       <c r="E56">
-        <f t="shared" ref="E56" si="57">SUM(D56:D58)</f>
+        <f t="shared" ref="E56" si="26">SUM(D56:D58)</f>
         <v>14</v>
       </c>
+      <c r="F56">
+        <v>6</v>
+      </c>
       <c r="G56">
-        <f t="shared" ref="G56:G60" si="58">VLOOKUP(A56, $S$12:$W$21, 4, FALSE)</f>
+        <f>VLOOKUP(A56, $S$12:$W$21, 4, FALSE)</f>
         <v>1.3</v>
       </c>
       <c r="K56">
-        <f t="shared" ref="K56:K62" si="59">VLOOKUP(A56, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A56, $S$12:$W$21, 3, FALSE)</f>
         <v>10</v>
       </c>
       <c r="M56">
-        <f t="shared" ref="M56:M59" si="60">VLOOKUP(A56, $S$12:$W$21, 2, FALSE)</f>
+        <f>VLOOKUP(A56, $S$12:$W$21, 2, FALSE)</f>
         <v>13</v>
       </c>
       <c r="O56">
-        <f t="shared" ref="O56:O59" si="61">$T$5</f>
+        <f t="shared" ref="O56:O59" si="27">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P56">
-        <f t="shared" ref="P56" si="62">O56*G56*E56</f>
+        <f>O56*G56*E56</f>
         <v>66.733333333333334</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q56">
+        <f>O56*M56*F56</f>
+        <v>286</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B57">
         <v>7</v>
@@ -1616,7 +1678,7 @@
         <v>10</v>
       </c>
       <c r="D57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="K57">
@@ -1624,9 +1686,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B58">
         <v>7</v>
@@ -1635,7 +1697,7 @@
         <v>12</v>
       </c>
       <c r="D58">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K58">
@@ -1643,9 +1705,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="Q61">
+        <f>O61*M61*F61</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>0</v>
@@ -1660,36 +1728,39 @@
         <v>6</v>
       </c>
       <c r="H70" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I70" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I70" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="J70" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K70" t="s">
         <v>9</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="M70" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N70" s="2" t="s">
-        <v>35</v>
+      <c r="N70" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="O70" t="s">
+        <v>17</v>
+      </c>
+      <c r="P70" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="P70" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q70" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B71">
         <v>3</v>
@@ -1732,7 +1803,8 @@
         <v>5</v>
       </c>
       <c r="N71">
-        <v>5</v>
+        <f>IF(ISBLANK(L71), J71*C71, L71)</f>
+        <v>0.50599520383693042</v>
       </c>
       <c r="O71">
         <f>$T$5</f>
@@ -1742,10 +1814,14 @@
         <f>O71*J71*E71</f>
         <v>11.131894484412468</v>
       </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q71">
+        <f>O71*N71*F71</f>
+        <v>1.8553157474020781</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B72">
         <v>3</v>
@@ -1754,17 +1830,17 @@
         <v>10</v>
       </c>
       <c r="D72">
-        <f t="shared" ref="D72:D73" si="63">IF(C72&lt;=K72, B72,0)</f>
+        <f t="shared" ref="D72:D73" si="28">IF(C72&lt;=K72, B72,0)</f>
         <v>3</v>
       </c>
       <c r="K72">
-        <f t="shared" ref="K72:K73" si="64">VLOOKUP(A72, $S$12:$W$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A72, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B73">
         <v>4</v>
@@ -1773,17 +1849,17 @@
         <v>12</v>
       </c>
       <c r="D73">
-        <f t="shared" si="63"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="K73">
-        <f t="shared" si="64"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A73, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B76">
         <v>3</v>
@@ -1818,11 +1894,12 @@
         <v>5.5</v>
       </c>
       <c r="M76">
-        <f t="shared" ref="M76" si="65">IF(ISBLANK(L76),VLOOKUP(A76, $S$12:$W$21, 2, FALSE),L76)</f>
+        <f>IF(ISBLANK(L76),VLOOKUP(A76, $S$12:$W$21, 2, FALSE),L76)</f>
         <v>5.5</v>
       </c>
       <c r="N76">
-        <v>5</v>
+        <f>IF(ISBLANK(L76), J76*C76, L76)</f>
+        <v>5.5</v>
       </c>
       <c r="O76">
         <f>$T$5</f>
@@ -1832,10 +1909,14 @@
         <f>O76*G76*E76</f>
         <v>12.1</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q76">
+        <f>O76*N76*F76</f>
+        <v>20.166666666666664</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B77">
         <v>3</v>
@@ -1844,17 +1925,17 @@
         <v>10</v>
       </c>
       <c r="D77">
-        <f t="shared" ref="D77:D78" si="66">IF(C77&lt;=K77, B77,0)</f>
+        <f t="shared" ref="D77:D78" si="29">IF(C77&lt;=K77, B77,0)</f>
         <v>3</v>
       </c>
       <c r="K77">
-        <f t="shared" ref="K77:K78" si="67">VLOOKUP(A77, $S$12:$W$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A77, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B78">
         <v>4</v>
@@ -1863,17 +1944,17 @@
         <v>12</v>
       </c>
       <c r="D78">
-        <f t="shared" si="66"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="K78">
-        <f t="shared" si="67"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A78, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B81">
         <v>3</v>
@@ -1916,7 +1997,8 @@
         <v>13</v>
       </c>
       <c r="N81">
-        <v>5</v>
+        <f>IF(ISBLANK(L81), J81*C81, L81)</f>
+        <v>2.8810810810810814</v>
       </c>
       <c r="O81">
         <f>$T$5</f>
@@ -1926,10 +2008,14 @@
         <f>O81*J81*E81</f>
         <v>63.383783783783784</v>
       </c>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q81">
+        <f>O81*N81*F81</f>
+        <v>10.563963963963964</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B82">
         <v>3</v>
@@ -1938,17 +2024,17 @@
         <v>10</v>
       </c>
       <c r="D82">
-        <f t="shared" ref="D82:D83" si="68">IF(C82&lt;=K82, B82,0)</f>
+        <f t="shared" ref="D82:D83" si="30">IF(C82&lt;=K82, B82,0)</f>
         <v>3</v>
       </c>
       <c r="K82">
-        <f t="shared" ref="K82:K83" si="69">VLOOKUP(A82, $S$12:$W$21, 3, FALSE)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A82, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B83">
         <v>4</v>
@@ -1957,17 +2043,17 @@
         <v>12</v>
       </c>
       <c r="D83">
-        <f t="shared" si="68"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="K83">
-        <f t="shared" si="69"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
+        <f>VLOOKUP(A83, $S$12:$W$21, 3, FALSE)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B86">
         <v>3</v>
@@ -2002,11 +2088,12 @@
         <v>4.5</v>
       </c>
       <c r="M86">
-        <f t="shared" ref="M86" si="70">IF(ISBLANK(L86),VLOOKUP(A86, $S$12:$W$21, 2, FALSE),L86)</f>
+        <f>IF(ISBLANK(L86),VLOOKUP(A86, $S$12:$W$21, 2, FALSE),L86)</f>
         <v>4.5</v>
       </c>
       <c r="N86">
-        <v>5</v>
+        <f>IF(ISBLANK(L86), J86*C86, L86)</f>
+        <v>4.5</v>
       </c>
       <c r="O86">
         <f>$T$5</f>
@@ -2016,10 +2103,14 @@
         <f>O86*G86*E86</f>
         <v>7.0714285714285712</v>
       </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q86">
+        <f>O86*N86*F86</f>
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B87">
         <v>3</v>
@@ -2028,17 +2119,17 @@
         <v>10</v>
       </c>
       <c r="D87">
-        <f t="shared" ref="D87:D88" si="71">IF(C87&lt;=K87, B87,0)</f>
+        <f t="shared" ref="D87:D88" si="31">IF(C87&lt;=K87, B87,0)</f>
         <v>0</v>
       </c>
       <c r="K87">
-        <f t="shared" ref="K87:K88" si="72">VLOOKUP(A87, $S$12:$W$21, 3, FALSE)</f>
+        <f>VLOOKUP(A87, $S$12:$W$21, 3, FALSE)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B88">
         <v>4</v>
@@ -2047,11 +2138,11 @@
         <v>12</v>
       </c>
       <c r="D88">
-        <f t="shared" si="71"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="K88">
-        <f t="shared" si="72"/>
+        <f>VLOOKUP(A88, $S$12:$W$21, 3, FALSE)</f>
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(calculators): responding to PR feedback, integrating new version of the chapter pdf
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/16-lulucf/16.5-lulucf.xlsx
+++ b/packages/calculators/src/modules/test/16-lulucf/16.5-lulucf.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/16-lulucf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1DA4E4-3AE5-6C4C-A792-58CF127D8BD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B7CF81-13F2-F94E-90C8-DA248FD3DFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51220" yWindow="11100" windowWidth="28800" windowHeight="26440" xr2:uid="{A7819E6E-1EF8-024D-B571-91DD1BC0E0B7}"/>
+    <workbookView xWindow="51200" yWindow="11100" windowWidth="28800" windowHeight="26440" xr2:uid="{A7819E6E-1EF8-024D-B571-91DD1BC0E0B7}"/>
   </bookViews>
   <sheets>
     <sheet name="16.5.1.1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="42">
   <si>
     <t>Act</t>
   </si>
@@ -209,15 +209,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -557,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{304E4C56-4465-6144-908F-761ED9C1F4A0}">
-  <dimension ref="A4:W88"/>
+  <dimension ref="A4:W91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="14.6640625" customWidth="1"/>
@@ -617,41 +613,38 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:23" s="6" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B9" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="4" t="s">
+    <row r="9" spans="1:23" s="4" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="B9" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="L9" s="5"/>
-      <c r="M9" s="4" t="s">
+      <c r="K9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N9" s="4"/>
+      <c r="N9" s="3"/>
     </row>
     <row r="10" spans="1:23" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -809,7 +802,7 @@
         <v>21</v>
       </c>
       <c r="T13">
-        <v>45</v>
+        <v>12.3</v>
       </c>
       <c r="U13">
         <v>15</v>
@@ -886,10 +879,10 @@
       </c>
       <c r="M16">
         <f>VLOOKUP(A16, $S$12:$W$21, 2, FALSE)</f>
-        <v>45</v>
+        <v>12.3</v>
       </c>
       <c r="O16">
-        <f t="shared" ref="O16:O59" si="3">$T$5</f>
+        <f t="shared" ref="O16" si="3">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P16">
@@ -1052,7 +1045,7 @@
         <v>9.6</v>
       </c>
       <c r="O21">
-        <f t="shared" ref="O21:O59" si="6">$T$5</f>
+        <f t="shared" ref="O21" si="6">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P21">
@@ -1151,7 +1144,7 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="O26">
-        <f t="shared" ref="O26:O59" si="9">$T$5</f>
+        <f t="shared" ref="O26" si="9">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P26">
@@ -1235,7 +1228,7 @@
         <v>5.2</v>
       </c>
       <c r="O31">
-        <f t="shared" ref="O31:O59" si="12">$T$5</f>
+        <f t="shared" ref="O31" si="12">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P31">
@@ -1319,7 +1312,7 @@
         <v>1.2</v>
       </c>
       <c r="O36">
-        <f t="shared" ref="O36:O59" si="15">$T$5</f>
+        <f t="shared" ref="O36" si="15">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P36">
@@ -1403,7 +1396,7 @@
         <v>1.5</v>
       </c>
       <c r="O41">
-        <f t="shared" ref="O41:O59" si="18">$T$5</f>
+        <f t="shared" ref="O41" si="18">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P41">
@@ -1487,7 +1480,7 @@
         <v>6.7</v>
       </c>
       <c r="O46">
-        <f t="shared" ref="O46:O59" si="21">$T$5</f>
+        <f t="shared" ref="O46" si="21">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P46">
@@ -1571,7 +1564,7 @@
         <v>6</v>
       </c>
       <c r="O51">
-        <f t="shared" ref="O51:O59" si="24">$T$5</f>
+        <f t="shared" ref="O51" si="24">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P51">
@@ -1655,7 +1648,7 @@
         <v>13</v>
       </c>
       <c r="O56">
-        <f t="shared" ref="O56:O59" si="27">$T$5</f>
+        <f t="shared" ref="O56" si="27">$T$5</f>
         <v>3.6666666666666665</v>
       </c>
       <c r="P56">
@@ -1706,13 +1699,91 @@
       </c>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>21</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+      <c r="D61">
+        <f t="shared" ref="D61:D65" si="28">IF(C61&lt;=K61, B61,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E61">
+        <f t="shared" ref="E61" si="29">SUM(D61:D63)</f>
+        <v>6</v>
+      </c>
+      <c r="F61">
+        <v>0.5</v>
+      </c>
+      <c r="G61">
+        <f>VLOOKUP(A61, $S$12:$W$21, 4, FALSE)</f>
+        <v>0.82</v>
+      </c>
+      <c r="K61">
+        <f>VLOOKUP(A61, $S$12:$W$21, 3, FALSE)</f>
+        <v>15</v>
+      </c>
+      <c r="M61">
+        <f>VLOOKUP(A61, $S$12:$W$21, 2, FALSE)</f>
+        <v>12.3</v>
+      </c>
+      <c r="O61">
+        <f t="shared" ref="O61" si="30">$T$5</f>
+        <v>3.6666666666666665</v>
+      </c>
+      <c r="P61">
+        <f>O61*G61*E61</f>
+        <v>18.04</v>
+      </c>
       <c r="Q61">
         <f>O61*M61*F61</f>
-        <v>0</v>
+        <v>22.55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>21</v>
+      </c>
+      <c r="B62">
+        <v>2</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
+      <c r="D62">
+        <f t="shared" si="28"/>
+        <v>2</v>
+      </c>
+      <c r="K62">
+        <f>VLOOKUP(A62, $S$12:$W$21, 3, FALSE)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>21</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63">
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <f t="shared" si="28"/>
+        <v>3</v>
+      </c>
+      <c r="K63">
+        <f>VLOOKUP(A63, $S$12:$W$21, 3, FALSE)</f>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:17" ht="34" x14ac:dyDescent="0.2">
-      <c r="A70" s="6" t="s">
+      <c r="A70" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B70" s="2" t="s">
@@ -1727,13 +1798,13 @@
       <c r="G70" t="s">
         <v>6</v>
       </c>
-      <c r="H70" s="5" t="s">
+      <c r="H70" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I70" s="4" t="s">
+      <c r="I70" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J70" s="5" t="s">
+      <c r="J70" s="4" t="s">
         <v>36</v>
       </c>
       <c r="K70" t="s">
@@ -1742,10 +1813,10 @@
       <c r="L70" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M70" s="3" t="s">
+      <c r="M70" t="s">
         <v>11</v>
       </c>
-      <c r="N70" s="3" t="s">
+      <c r="N70" t="s">
         <v>41</v>
       </c>
       <c r="O70" t="s">
@@ -1830,7 +1901,7 @@
         <v>10</v>
       </c>
       <c r="D72">
-        <f t="shared" ref="D72:D73" si="28">IF(C72&lt;=K72, B72,0)</f>
+        <f t="shared" ref="D72:D73" si="31">IF(C72&lt;=K72, B72,0)</f>
         <v>3</v>
       </c>
       <c r="K72">
@@ -1849,7 +1920,7 @@
         <v>12</v>
       </c>
       <c r="D73">
-        <f t="shared" si="28"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="K73">
@@ -1925,7 +1996,7 @@
         <v>10</v>
       </c>
       <c r="D77">
-        <f t="shared" ref="D77:D78" si="29">IF(C77&lt;=K77, B77,0)</f>
+        <f t="shared" ref="D77:D78" si="32">IF(C77&lt;=K77, B77,0)</f>
         <v>3</v>
       </c>
       <c r="K77">
@@ -1944,7 +2015,7 @@
         <v>12</v>
       </c>
       <c r="D78">
-        <f t="shared" si="29"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="K78">
@@ -2024,7 +2095,7 @@
         <v>10</v>
       </c>
       <c r="D82">
-        <f t="shared" ref="D82:D83" si="30">IF(C82&lt;=K82, B82,0)</f>
+        <f t="shared" ref="D82:D83" si="33">IF(C82&lt;=K82, B82,0)</f>
         <v>3</v>
       </c>
       <c r="K82">
@@ -2043,7 +2114,7 @@
         <v>12</v>
       </c>
       <c r="D83">
-        <f t="shared" si="30"/>
+        <f t="shared" si="33"/>
         <v>0</v>
       </c>
       <c r="K83">
@@ -2119,7 +2190,7 @@
         <v>10</v>
       </c>
       <c r="D87">
-        <f t="shared" ref="D87:D88" si="31">IF(C87&lt;=K87, B87,0)</f>
+        <f t="shared" ref="D87:D88" si="34">IF(C87&lt;=K87, B87,0)</f>
         <v>0</v>
       </c>
       <c r="K87">
@@ -2138,13 +2209,16 @@
         <v>12</v>
       </c>
       <c r="D88">
-        <f t="shared" si="31"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="K88">
         <f>VLOOKUP(A88, $S$12:$W$21, 3, FALSE)</f>
         <v>7</v>
       </c>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="I91" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>